<commit_message>
Refresh application visual design
</commit_message>
<xml_diff>
--- a/config/templates/OAS-K_Configuration_Template v.1.xlsx
+++ b/config/templates/OAS-K_Configuration_Template v.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Project\OfficeAutomationSuite-Karina\config\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EA413D-D151-4C7C-BE72-8631F15F8A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DCF62D-5F3E-4903-B594-317FDDBE657B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guide" sheetId="1" r:id="rId1"/>
@@ -3605,7 +3605,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="11">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3669,20 +3676,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4233,7 +4226,8 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="4" width="14" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" customWidth="1"/>
+    <col min="2" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1">
@@ -17176,13 +17170,13 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="duplicateValues" dxfId="9" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I4">
-    <cfRule type="expression" dxfId="9" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>I4="FALSE"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih nilai dari daftar yang tersedia." promptTitle="OAS-K" prompt="Gunakan salah satu nilai yang tersedia." sqref="I4" xr:uid="{00000000-0002-0000-0500-000000000000}">

</xml_diff>